<commit_message>
CU updates, Daily log complete, CST update
Updated the CU adding structure and MC0, partially updated the CST to reflect the new design direction, and completed the daily log for 6/4
</commit_message>
<xml_diff>
--- a/Design_Docs/RISC-V_CST.xlsx
+++ b/Design_Docs/RISC-V_CST.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Apex\Projects\RISC-V_Project\sfm_RISC-V\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Apex\Projects\RISC-V_Project\sfm_RISC-V\Design_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7C3C8B-66B4-465E-A7A8-AE3FCEECB894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{474280B4-CC3D-4DFB-81F3-6B1E2FA5775C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="45972" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="44">
   <si>
     <t>MC\CS</t>
   </si>
@@ -154,13 +154,16 @@
   </si>
   <si>
     <t>PCout</t>
+  </si>
+  <si>
+    <t>May not need</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -174,13 +177,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -195,10 +210,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -614,46 +632,48 @@
       <c r="N3" s="1"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="M4" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="N4" s="1"/>
+      <c r="N4" s="1" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">

</xml_diff>